<commit_message>
List block: resolve AEM /content page paths; replace homepage I want to block
- list.js resolves page links picked in Universal Editor
  (/content/icare-migration-demo/<path>.html) to the page's address where the
  block is shown: /<path> on the published site, unchanged in Universal
  Editor, /content/<path> in the local preview. DAM assets, normal paths and
  external links are left as they are. Untitled links still show the linked
  page's title.
- Homepage importer: the list block now replaces the columns-links
  "I want to..." block in the same section (heading kept as default content).
  Internal links are authored as untitled /content page paths; external portal
  links keep the source text as their title.
- list.css: section spacing of the source "I want to..." section.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","search-banner","cards-audience","columns-links","list","columns-campaign","columns-story","cards-news","cards-resources"]</t>
+    <t>["hero","search-banner","cards-audience","list","columns-campaign","columns-story","cards-news","cards-resources"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-20T20:06:55.385Z</t>
+    <t>2026-10-20T20:41:36.322Z</t>
   </si>
   <si>
     <t>Insurance and Care NSW | icare</t>

</xml_diff>

<commit_message>
Add news-listing block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 24
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","search-banner","cards-audience","list","columns-campaign","columns-story","cards-news","cards-resources"]</t>
+    <t>["hero","search-banner","cards-audience","list","columns-campaign","columns-story","news-listing","cards-resources"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-21T01:44:42.721Z</t>
+    <t>2026-10-28T11:22:51.797Z</t>
   </si>
   <si>
     <t>Insurance and Care NSW | icare</t>
@@ -133,7 +133,7 @@
     <t>workers-compensation/employers</t>
   </si>
   <si>
-    <t>2026-10-20T22:26:56.105Z</t>
+    <t>2026-10-21T01:46:53.801Z</t>
   </si>
   <si>
     <t>Employers | icare</t>
@@ -154,7 +154,7 @@
     <t>section-overview-hub</t>
   </si>
   <si>
-    <t>2026-10-20T22:26:30.758Z</t>
+    <t>2026-10-28T10:25:58.570Z</t>
   </si>
   <si>
     <t>Small business hub | icare</t>
@@ -175,7 +175,7 @@
     <t>hero-image-content-with-sidebar</t>
   </si>
   <si>
-    <t>2026-10-20T22:26:41.952Z</t>
+    <t>2026-10-28T10:26:10.651Z</t>
   </si>
   <si>
     <t>Notify us of an injury or make a claim | icare</t>
@@ -196,7 +196,7 @@
     <t>news-story-with-video</t>
   </si>
   <si>
-    <t>2026-10-21T01:28:41.607Z</t>
+    <t>2026-10-28T11:20:15.262Z</t>
   </si>
   <si>
     <t>Adaptive sports helps Jarrod reimagine whats possible | icare</t>
@@ -214,7 +214,7 @@
     <t>news-and-stories/2024/annabelle-shares-her-passion-for-adaptive-sports</t>
   </si>
   <si>
-    <t>2026-10-21T01:28:50.004Z</t>
+    <t>2026-10-28T11:21:08.929Z</t>
   </si>
   <si>
     <t>Annabelle shares her passion for adaptive sports | icare</t>
@@ -229,7 +229,7 @@
     <t>news-and-stories/2024/reimagining-your-life</t>
   </si>
   <si>
-    <t>2026-10-21T01:29:44.286Z</t>
+    <t>2026-10-28T11:22:02.720Z</t>
   </si>
   <si>
     <t>Reimagining your life | icare</t>
@@ -247,7 +247,7 @@
     <t>news-and-stories/2024/shine-magazine-summer-2024-edition-is-out-now</t>
   </si>
   <si>
-    <t>2026-10-21T01:29:55.301Z</t>
+    <t>2026-10-28T11:22:11.869Z</t>
   </si>
   <si>
     <t>Shine Magazine summer 2024 edition is out now | icare</t>
@@ -265,7 +265,7 @@
     <t>news-and-stories/2025/icare-safeguards-nsw-workers-with-new-lung-health-mobile-clinic</t>
   </si>
   <si>
-    <t>2026-10-21T01:30:07.156Z</t>
+    <t>2026-10-28T11:22:21.856Z</t>
   </si>
   <si>
     <t>icare safeguards NSW workers with new Lung Health Mobile Clinic | icare</t>
@@ -286,7 +286,7 @@
     <t>guide-with-page-nav</t>
   </si>
   <si>
-    <t>2026-10-20T03:54:50.094Z</t>
+    <t>2026-10-28T10:15:08.989Z</t>
   </si>
   <si>
     <t>Apprentice Incentive Scheme | icare</t>
@@ -304,7 +304,7 @@
     <t>workers-compensation/employers/classifying-your-workers</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:00.589Z</t>
+    <t>2026-10-28T10:15:17.307Z</t>
   </si>
   <si>
     <t>Classifying Workers or Contractors for Workers Compensation | icare</t>
@@ -319,7 +319,7 @@
     <t>workers-compensation/employers/forms-and-resources</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:08.559Z</t>
+    <t>2026-10-28T10:15:28.071Z</t>
   </si>
   <si>
     <t>Forms and resources | icare</t>
@@ -337,7 +337,7 @@
     <t>workers-compensation/employers/how-much-will-it-cost</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:17.699Z</t>
+    <t>2026-10-28T10:15:36.212Z</t>
   </si>
   <si>
     <t>Costs and premiums | icare</t>
@@ -355,7 +355,7 @@
     <t>workers-compensation/employers/insurance-for-related-businesses</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:26.791Z</t>
+    <t>2026-10-28T10:15:45.768Z</t>
   </si>
   <si>
     <t>What is Grouping Insurance for Related Businesses? | icare</t>
@@ -415,7 +415,7 @@
     <t>workers-compensation/employers/understanding-icare-and-workers-compensation</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:04.735Z</t>
+    <t>2026-10-28T10:24:09.532Z</t>
   </si>
   <si>
     <t>Understanding ​​icare and Workers Compensation | icare</t>
@@ -433,7 +433,7 @@
     <t>workers-compensation/employers/whats-covered</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:15.887Z</t>
+    <t>2026-10-28T10:24:17.285Z</t>
   </si>
   <si>
     <t>Whats covered | icare</t>
@@ -448,7 +448,7 @@
     <t>workers-compensation/employers/whats-new</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:24.946Z</t>
+    <t>2026-10-28T10:24:25.656Z</t>
   </si>
   <si>
     <t>What's new in Workers Compensation | icare</t>
@@ -463,7 +463,7 @@
     <t>workers-compensation/employers/who-needs-a-policy</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:36.687Z</t>
+    <t>2026-10-28T10:24:38.662Z</t>
   </si>
   <si>
     <t>Who needs a policy | icare</t>
@@ -481,7 +481,7 @@
     <t>workers-compensation/employers/workers-compensation-reform-faqs</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:44.393Z</t>
+    <t>2026-10-28T10:24:48.165Z</t>
   </si>
   <si>
     <t>Workers Compensation Reform FAQs | icare</t>
@@ -496,7 +496,7 @@
     <t>workers-compensation/employers/your-responsibilities-as-an-employer</t>
   </si>
   <si>
-    <t>2026-10-20T04:02:51.736Z</t>
+    <t>2026-10-28T10:24:56.712Z</t>
   </si>
   <si>
     <t>Your responsibilities | icare</t>
@@ -532,7 +532,7 @@
     <t>workers-compensation/employers/manage-your-policy/cancel-your-workers-insurance-policy</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:39.086Z</t>
+    <t>2026-10-28T10:15:57.349Z</t>
   </si>
   <si>
     <t>Cancel your workers insurance policy | icare</t>
@@ -550,7 +550,7 @@
     <t>workers-compensation/employers/manage-your-policy/declaring-wages</t>
   </si>
   <si>
-    <t>2026-10-20T03:54:39.837Z</t>
+    <t>2026-10-28T10:14:58.989Z</t>
   </si>
   <si>
     <t>Declaring Wages to Calculate Workers Compensation premiums | icare</t>
@@ -565,7 +565,7 @@
     <t>workers-compensation/employers/manage-your-policy/download-a-certificate-of-currency</t>
   </si>
   <si>
-    <t>2026-10-20T03:55:50.169Z</t>
+    <t>2026-10-28T10:16:04.939Z</t>
   </si>
   <si>
     <t>Download a Certificate of Currency | icare</t>
@@ -580,7 +580,7 @@
     <t>workers-compensation/employers/manage-your-policy/faqs-wage-audit-process</t>
   </si>
   <si>
-    <t>2026-10-20T03:56:03.695Z</t>
+    <t>2026-10-28T10:16:16.504Z</t>
   </si>
   <si>
     <t>FAQs Wage Audit Process | icare</t>
@@ -595,7 +595,7 @@
     <t>workers-compensation/employers/manage-your-policy/how-to-access-your-monthly-cost-of-claims-report</t>
   </si>
   <si>
-    <t>2026-10-20T03:56:10.422Z</t>
+    <t>2026-10-28T10:16:29.612Z</t>
   </si>
   <si>
     <t>How to access your monthly Cost of Claims report | icare</t>
@@ -610,7 +610,7 @@
     <t>workers-compensation/employers/manage-your-policy/premium-disputes</t>
   </si>
   <si>
-    <t>2026-10-20T03:56:22.400Z</t>
+    <t>2026-10-28T10:16:39.069Z</t>
   </si>
   <si>
     <t>Premium disputes | icare</t>
@@ -625,7 +625,7 @@
     <t>workers-compensation/employers/manage-your-policy/renew-your-policy</t>
   </si>
   <si>
-    <t>2026-10-20T22:28:02.655Z</t>
+    <t>2026-10-28T10:17:32.428Z</t>
   </si>
   <si>
     <t>Renew your Workers Insurance policy | icare</t>
@@ -640,7 +640,7 @@
     <t>workers-compensation/employers/manage-your-policy/update-your-policy-details</t>
   </si>
   <si>
-    <t>2026-10-20T03:57:28.007Z</t>
+    <t>2026-10-28T10:17:45.308Z</t>
   </si>
   <si>
     <t>Update your policy details | icare</t>
@@ -655,7 +655,7 @@
     <t>workers-compensation/employers/new-policy/2026-premium-rate-freeze</t>
   </si>
   <si>
-    <t>2026-10-20T03:57:41.380Z</t>
+    <t>2026-10-28T10:17:57.660Z</t>
   </si>
   <si>
     <t>2026 Premium Rate Freeze | icare</t>
@@ -670,7 +670,7 @@
     <t>workers-compensation/employers/new-policy/claims-performance-adjustment-rates</t>
   </si>
   <si>
-    <t>2026-10-20T03:57:52.559Z</t>
+    <t>2026-10-28T10:18:09.118Z</t>
   </si>
   <si>
     <t>Claims performance adjustment rates | icare</t>
@@ -688,7 +688,7 @@
     <t>workers-compensation/employers/new-policy/how-to-lower-your-premium</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:02.333Z</t>
+    <t>2026-10-28T10:18:19.429Z</t>
   </si>
   <si>
     <t>How to lower your premium | icare</t>
@@ -703,7 +703,7 @@
     <t>workers-compensation/employers/new-policy/how-to-pay-your-premium</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:10.843Z</t>
+    <t>2026-10-28T10:18:32.284Z</t>
   </si>
   <si>
     <t>How to pay your premium | icare</t>
@@ -718,7 +718,7 @@
     <t>workers-compensation/employers/new-policy/loss-prevention-and-recovery</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:18.715Z</t>
+    <t>2026-10-28T10:18:41.251Z</t>
   </si>
   <si>
     <t>Loss Prevention and Recovery Products for Calculating Premium | icare</t>
@@ -733,7 +733,7 @@
     <t>workers-compensation/employers/new-policy/multiple-business-activities-and-wic-classification</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:30.386Z</t>
+    <t>2026-10-28T10:18:54.391Z</t>
   </si>
   <si>
     <t>Multiple business activities and WIC classification | icare</t>
@@ -751,7 +751,7 @@
     <t>workers-compensation/employers/new-policy/premium-calculation-experience-rated</t>
   </si>
   <si>
-    <t>2026-10-20T22:27:10.353Z</t>
+    <t>2026-10-28T10:19:06.023Z</t>
   </si>
   <si>
     <t>Premium calculation experience-rated | icare</t>
@@ -769,7 +769,7 @@
     <t>workers-compensation/employers/new-policy/premium-calculation-for-small-employers</t>
   </si>
   <si>
-    <t>2026-10-20T03:58:55.911Z</t>
+    <t>2026-10-28T10:19:18.644Z</t>
   </si>
   <si>
     <t>Premium calculation for small employers | icare</t>
@@ -784,7 +784,7 @@
     <t>workers-compensation/employers/new-policy/take-out-a-policy</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:07.318Z</t>
+    <t>2026-10-28T10:19:39.345Z</t>
   </si>
   <si>
     <t>Take out a policy | icare</t>
@@ -802,7 +802,7 @@
     <t>workers-compensation/employers/new-policy/understanding-wics-and-premium-rates</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:19.064Z</t>
+    <t>2026-10-28T10:19:51.263Z</t>
   </si>
   <si>
     <t>Understanding WICS and premium rates | icare</t>
@@ -817,7 +817,7 @@
     <t>workers-compensation/employers/new-policy/understanding-your-cover</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:31.385Z</t>
+    <t>2026-10-28T10:20:03.027Z</t>
   </si>
   <si>
     <t>Understanding your cover | icare</t>
@@ -835,7 +835,7 @@
     <t>workers-compensation/employers/new-policy/understanding-your-premium</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:42.489Z</t>
+    <t>2026-10-28T10:20:14.827Z</t>
   </si>
   <si>
     <t>Understanding your premium | icare</t>
@@ -853,7 +853,7 @@
     <t>workers-compensation/employers/new-policy/what-is-premium-capping-and-how-does-it-work</t>
   </si>
   <si>
-    <t>2026-10-20T03:59:53.640Z</t>
+    <t>2026-10-28T10:20:24.496Z</t>
   </si>
   <si>
     <t>What is premium capping and how does it work? | icare</t>
@@ -871,7 +871,7 @@
     <t>workers-compensation/employers/prevention-and-education/adssi-limited</t>
   </si>
   <si>
-    <t>2026-10-20T22:22:12.553Z</t>
+    <t>2026-10-28T10:20:34.243Z</t>
   </si>
   <si>
     <t>ADSSI Limited | icare</t>
@@ -889,7 +889,7 @@
     <t>workers-compensation/employers/prevention-and-education/asbjv</t>
   </si>
   <si>
-    <t>2026-10-20T22:22:20.748Z</t>
+    <t>2026-10-28T10:20:42.143Z</t>
   </si>
   <si>
     <t>ASBJV | icare</t>
@@ -904,7 +904,7 @@
     <t>workers-compensation/employers/prevention-and-education/ebos-group</t>
   </si>
   <si>
-    <t>2026-10-20T22:22:29.134Z</t>
+    <t>2026-10-28T10:21:35.670Z</t>
   </si>
   <si>
     <t>EBOS Group | icare</t>
@@ -922,7 +922,7 @@
     <t>workers-compensation/employers/prevention-and-education/expert-consultation</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:25.683Z</t>
+    <t>2026-10-28T10:21:43.977Z</t>
   </si>
   <si>
     <t>Expert consultation | icare</t>
@@ -937,7 +937,7 @@
     <t>workers-compensation/employers/prevention-and-education/injury-prevention-resource-hub</t>
   </si>
   <si>
-    <t>2026-10-20T04:03:03.005Z</t>
+    <t>2026-10-28T10:25:04.443Z</t>
   </si>
   <si>
     <t>Injury prevention resource hub | icare</t>
@@ -955,7 +955,7 @@
     <t>workers-compensation/employers/prevention-and-education/injury-prevention</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:35.785Z</t>
+    <t>2026-10-28T10:21:54.242Z</t>
   </si>
   <si>
     <t>Injury Prevention | icare</t>
@@ -970,7 +970,7 @@
     <t>workers-compensation/employers/prevention-and-education/metcash</t>
   </si>
   <si>
-    <t>2026-10-20T22:23:22.286Z</t>
+    <t>2026-10-28T10:22:47.893Z</t>
   </si>
   <si>
     <t>Metcash | icare</t>
@@ -985,7 +985,7 @@
     <t>workers-compensation/employers/prevention-and-education/the-safety-locker</t>
   </si>
   <si>
-    <t>2026-10-20T04:00:52.169Z</t>
+    <t>2026-10-28T10:22:55.542Z</t>
   </si>
   <si>
     <t>The safety locker | icare</t>
@@ -1000,7 +1000,7 @@
     <t>workers-compensation/employers/prevention-and-education/training-programs</t>
   </si>
   <si>
-    <t>2026-10-20T04:01:01.339Z</t>
+    <t>2026-10-28T10:23:02.915Z</t>
   </si>
   <si>
     <t>Training programs | icare</t>
@@ -1018,7 +1018,7 @@
     <t>workers-compensation/employers/prevention-and-education/weathertex</t>
   </si>
   <si>
-    <t>2026-10-20T22:24:16.095Z</t>
+    <t>2026-10-28T10:23:55.650Z</t>
   </si>
   <si>
     <t>Weathertex | icare</t>

</xml_diff>